<commit_message>
Auto: Week 26/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W26_2026.xlsx
+++ b/Gulf_Dashboard_W26_2026.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -739,12 +739,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>PRJ-009</t>
+          <t>PRJ-008</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>AL1 (Alpha 1)</t>
+          <t>GULF AC8</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -758,12 +758,12 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>PRJ-010</t>
+          <t>PRJ-009</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>AL2 (Alpha 2)</t>
+          <t>AL1 (Alpha 1)</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -777,12 +777,12 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>PRJ-011</t>
+          <t>PRJ-010</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>ECE</t>
+          <t>AL2 (Alpha 2)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -794,22 +794,60 @@
       <c r="E11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>PRJ-011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>ECE</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>PRJ-012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>GULF_Wayu</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>PRJ-013</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>GCE</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Details regarding the routingconnecttoTransformerwerenot found.
 There are routing conflicts in the STG building cable layout.
@@ -833,7 +871,7 @@
 6 Coordinate to participate in community activities and related -School ,Government As CR -</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Commissioning 0.00% 0.00% -
 Key Lookahead milestone:
@@ -858,23 +896,23 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>PRJ-014</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>GSE</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Delay finish of bunker foundations up to ground level. Target on PMS 07 May 2026.
 Delay finish of STG foundations up to ground level. Target on PMS 25 May 2026.
@@ -898,7 +936,7 @@
 - Request to EPC to catch up plan. Increase man power.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Activities CC/SC (*)
 Plan% Actual% Diff.% Plan% Actual% Diff.% Acc. Plan%
@@ -923,23 +961,23 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>PRJ-015</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>KKE</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>311-314 Refuse Bunker Super structure up to 35.5m elevation 9 May 26 23 Nov 26 Delay Start
 325-326 Tipping hall Foundation up to ground (Include piling work) 1 Feb 26 9 Jul 26 8 Feb 26 On going
@@ -963,7 +1001,7 @@
 No Safety Sign ‘Confined space’</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Catch-up plan of STG &amp; ECB: for partial hand over include all activities required to achieve Back
 Energization on 21-Dec-2026 is under review by CEEC and expected to be submitted next week
@@ -988,23 +1026,23 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>PRJ-016</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>MKP</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Bunker Pit Wall to +5.45 EL
 Bunker Building ground level construction
@@ -1028,7 +1066,7 @@
 2 Request CEEC to update purchasing status of Duct bank and Cathodic protection.</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>(26 Jun 26) (03 Jul 26)
 Activities CC/SC (*)
@@ -1053,23 +1091,23 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>PRJ-017</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>MPE</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>248 Incinerator Arrival at site 21 May 26 28 May 26 Delayed Planned delivery to site on 11/07
 253 Steam turbine Arrivalat site 22 Dec 26 29 Dec 26
@@ -1093,7 +1131,7 @@
 activities and related government agencies appropriate.</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Key Lookahead milestone:
 Pre-conditions required: None
@@ -1118,23 +1156,23 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>PRJ-018</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>PFP</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Tasks that have started and those that have not yet started are behind schedule (PMS plan)
 Safety Weekly Audit issue status by weekly
@@ -1158,7 +1196,7 @@
 Concern area of EPC/STECON</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Key Lookahead milestone:
 Total Man-Hours 129,797 Pre-conditions required:
@@ -1183,23 +1221,23 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>PRJ-019</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>PKP</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>FGT &amp; STG Civil Work : Level 3 schedule update from CEEC is still pending.
 Limited site access roads may impact construction productivity and material logistics.
@@ -1223,7 +1261,7 @@
 Closed 0 issues</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>TRIR 0 3. Catch-up plan for the partial handover of the FGT area, to HUASI erection work is under review by
 CEEC and expected to be submitted next week
@@ -1248,23 +1286,23 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>PRJ-020</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>PSD</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Bunker, Boiler, FGT &amp; STG Civil work : The Level 3 schedule update from CEEC is still pending. CEEC has committed to submitting the schedule next week
 Bunker Wall Deviation: Corrective modification to be processed via FCN.Bunker pit volume reduced by ~0.12% (negligible impact).
@@ -1288,7 +1326,7 @@
 ▪ PEA ดำ เนินกำรเรอื งเอกสำรของและเตรยี มทมี ส ำหรบั ทำ งำน ใชเ้วลำโดยประมำณ 1-2 เดอื น</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Jun 2026) Jul 2026)
 Activities CC/SC (*)
@@ -1313,23 +1351,23 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>PRJ-021</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>PWW1</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Back Energize Work
 Retaining wall (PWW1, 2) - Final drawing
@@ -1353,7 +1391,7 @@
 Since 2 Apr 2026</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Safety &amp; Health:
 • Safety Toolbox Talk before starting work and Mass Safety Talk.
@@ -1378,23 +1416,23 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>PRJ-022</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>PWW2</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Refuse Bunker foundation construction work
 Boiler Island foundation construction
@@ -1418,7 +1456,7 @@
 Follow up equipment(Jockey water pump and Diesel water pump). [Now status CEEC Bidding Process]</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Safety &amp; Health:
 • Safety Toolbox Talk before starting work and Mass Safety Talk.
@@ -1443,23 +1481,23 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>PRJ-023</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>TPP</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Bunker Pit Wall to +8.00 EL
 Bunker Building ground level construction
@@ -1483,7 +1521,7 @@
 STECON clarified that the work will catch up with the working plan at the floor EL +4.25m activity.</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>(26 Jun 26) (03 Jul 26)
 Activities CC/SC (*)
@@ -1508,23 +1546,23 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>PRJ-024</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>TSE</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Delay finish of bunker foundations up to ground level. Target on PMS 08 May 2026.
 Delay finish of STG foundations up to ground level. Target on PMS 08 Jun 2026.
@@ -1548,7 +1586,7 @@
 IWTE–TSE–NCR–C–003 21/04/2026 Civil Honey combing and voids were identified after formwork removal waste bunker column TSE . Open</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Activities CC/SC (*)
 Plan% Actual% Diff.% Plan% Actual% Diff.% Acc. Plan%
@@ -1573,23 +1611,23 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>PRJ-025</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Pak Lay</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>No. Description Progress Remark
 Contractor submitted the Contracor’s
@@ -1613,7 +1651,7 @@
 8 material supply EPC Immediate</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>List of Issues to be Coordinated
 shall follow this
@@ -1638,23 +1676,23 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>PRJ-026</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Pak Beng</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Right bank abutment、
 Downstream Approach
@@ -1678,7 +1716,7 @@
 defective areas and corrective works.</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Health and Safety Health and Safety
 - Ongoing conduct HSE general induction and training for
@@ -1703,24 +1741,24 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>PRJ-027</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>TTT</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>